<commit_message>
Add standard terms playbook and customer service, design, finance, legal, and HR hands-on lab sessions
- Created `AcmeBottling_Standard_Terms.md` for standard contract language reference.
- Added `MS-4004.X_Customer_Service.md` for customer service hands-on lab.
- Introduced `MS-4004.X_Design_and_Engineering.md` for design and engineering hands-on lab.
- Updated finance session to reference new file names for monthly actuals and AR aging sheets.
- Added `MS-4004.X_Legal.md` for legal hands-on lab focusing on contract review.
- Updated HR session to reference new file names for role description, onboarding notes, skills list, and communication brief.
</commit_message>
<xml_diff>
--- a/data/AcmeBottling_Master_Reference.xlsx
+++ b/data/AcmeBottling_Master_Reference.xlsx
@@ -12,13 +12,14 @@
     <sheet name="Suppliers" sheetId="3" r:id="rId3"/>
     <sheet name="Inventory" sheetId="4" r:id="rId4"/>
     <sheet name="Orders" sheetId="5" r:id="rId5"/>
+    <sheet name="Opportunities" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="377">
   <si>
     <t>CustomerID</t>
   </si>
@@ -822,6 +823,333 @@
   </si>
   <si>
     <t>QA reinspection</t>
+  </si>
+  <si>
+    <t>OpportunityID</t>
+  </si>
+  <si>
+    <t>Stage</t>
+  </si>
+  <si>
+    <t>CreatedDate</t>
+  </si>
+  <si>
+    <t>LastActivityDate</t>
+  </si>
+  <si>
+    <t>AgeDays</t>
+  </si>
+  <si>
+    <t>EstValueUSD</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>OPP-7001</t>
+  </si>
+  <si>
+    <t>OPP-7002</t>
+  </si>
+  <si>
+    <t>OPP-7003</t>
+  </si>
+  <si>
+    <t>OPP-7004</t>
+  </si>
+  <si>
+    <t>OPP-7005</t>
+  </si>
+  <si>
+    <t>OPP-7006</t>
+  </si>
+  <si>
+    <t>OPP-7007</t>
+  </si>
+  <si>
+    <t>OPP-7008</t>
+  </si>
+  <si>
+    <t>OPP-7009</t>
+  </si>
+  <si>
+    <t>OPP-7010</t>
+  </si>
+  <si>
+    <t>OPP-7011</t>
+  </si>
+  <si>
+    <t>OPP-7012</t>
+  </si>
+  <si>
+    <t>OPP-7013</t>
+  </si>
+  <si>
+    <t>OPP-7014</t>
+  </si>
+  <si>
+    <t>OPP-7015</t>
+  </si>
+  <si>
+    <t>OPP-7016</t>
+  </si>
+  <si>
+    <t>OPP-7017</t>
+  </si>
+  <si>
+    <t>OPP-7018</t>
+  </si>
+  <si>
+    <t>OPP-7019</t>
+  </si>
+  <si>
+    <t>OPP-7020</t>
+  </si>
+  <si>
+    <t>OPP-7021</t>
+  </si>
+  <si>
+    <t>OPP-7022</t>
+  </si>
+  <si>
+    <t>OPP-7023</t>
+  </si>
+  <si>
+    <t>OPP-7024</t>
+  </si>
+  <si>
+    <t>OPP-7025</t>
+  </si>
+  <si>
+    <t>OPP-7026</t>
+  </si>
+  <si>
+    <t>OPP-7027</t>
+  </si>
+  <si>
+    <t>OPP-7028</t>
+  </si>
+  <si>
+    <t>OPP-7029</t>
+  </si>
+  <si>
+    <t>OPP-7030</t>
+  </si>
+  <si>
+    <t>OPP-7031</t>
+  </si>
+  <si>
+    <t>OPP-7032</t>
+  </si>
+  <si>
+    <t>OPP-7033</t>
+  </si>
+  <si>
+    <t>OPP-7034</t>
+  </si>
+  <si>
+    <t>OPP-7035</t>
+  </si>
+  <si>
+    <t>OPP-7036</t>
+  </si>
+  <si>
+    <t>OPP-7037</t>
+  </si>
+  <si>
+    <t>OPP-7038</t>
+  </si>
+  <si>
+    <t>OPP-7039</t>
+  </si>
+  <si>
+    <t>OPP-7040</t>
+  </si>
+  <si>
+    <t>OPP-7041</t>
+  </si>
+  <si>
+    <t>OPP-7042</t>
+  </si>
+  <si>
+    <t>OPP-7043</t>
+  </si>
+  <si>
+    <t>OPP-7044</t>
+  </si>
+  <si>
+    <t>OPP-7045</t>
+  </si>
+  <si>
+    <t>Proposal</t>
+  </si>
+  <si>
+    <t>Lost</t>
+  </si>
+  <si>
+    <t>Qualifying</t>
+  </si>
+  <si>
+    <t>Won</t>
+  </si>
+  <si>
+    <t>Negotiation</t>
+  </si>
+  <si>
+    <t>2026-02-19</t>
+  </si>
+  <si>
+    <t>2026-03-03</t>
+  </si>
+  <si>
+    <t>2026-07-06</t>
+  </si>
+  <si>
+    <t>2026-05-18</t>
+  </si>
+  <si>
+    <t>2026-04-11</t>
+  </si>
+  <si>
+    <t>2026-06-09</t>
+  </si>
+  <si>
+    <t>2026-04-12</t>
+  </si>
+  <si>
+    <t>2026-07-13</t>
+  </si>
+  <si>
+    <t>2026-06-20</t>
+  </si>
+  <si>
+    <t>2026-05-24</t>
+  </si>
+  <si>
+    <t>2026-02-21</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>2026-02-03</t>
+  </si>
+  <si>
+    <t>2026-04-16</t>
+  </si>
+  <si>
+    <t>2026-03-10</t>
+  </si>
+  <si>
+    <t>2026-04-27</t>
+  </si>
+  <si>
+    <t>2026-05-07</t>
+  </si>
+  <si>
+    <t>2026-02-11</t>
+  </si>
+  <si>
+    <t>2026-06-21</t>
+  </si>
+  <si>
+    <t>2026-04-08</t>
+  </si>
+  <si>
+    <t>2026-05-26</t>
+  </si>
+  <si>
+    <t>2026-07-08</t>
+  </si>
+  <si>
+    <t>2026-01-29</t>
+  </si>
+  <si>
+    <t>2026-05-14</t>
+  </si>
+  <si>
+    <t>2026-04-29</t>
+  </si>
+  <si>
+    <t>2026-03-18</t>
+  </si>
+  <si>
+    <t>2026-03-07</t>
+  </si>
+  <si>
+    <t>2026-05-25</t>
+  </si>
+  <si>
+    <t>2026-03-21</t>
+  </si>
+  <si>
+    <t>2026-04-15</t>
+  </si>
+  <si>
+    <t>2026-07-22</t>
+  </si>
+  <si>
+    <t>2026-02-14</t>
+  </si>
+  <si>
+    <t>2026-04-19</t>
+  </si>
+  <si>
+    <t>2026-08-03</t>
+  </si>
+  <si>
+    <t>2026-01-26</t>
+  </si>
+  <si>
+    <t>2026-03-13</t>
+  </si>
+  <si>
+    <t>2026-05-16</t>
+  </si>
+  <si>
+    <t>2026-04-05</t>
+  </si>
+  <si>
+    <t>2026-07-19</t>
+  </si>
+  <si>
+    <t>2026-04-17</t>
+  </si>
+  <si>
+    <t>2026-06-18</t>
+  </si>
+  <si>
+    <t>2026-05-28</t>
+  </si>
+  <si>
+    <t>2026-05-05</t>
+  </si>
+  <si>
+    <t>2026-06-19</t>
+  </si>
+  <si>
+    <t>2026-07-05</t>
+  </si>
+  <si>
+    <t>2026-05-21</t>
+  </si>
+  <si>
+    <t>2026-06-05</t>
+  </si>
+  <si>
+    <t>2026-07-02</t>
+  </si>
+  <si>
+    <t>2026-06-26</t>
+  </si>
+  <si>
+    <t>2026-05-04</t>
+  </si>
+  <si>
+    <t>2026-05-11</t>
+  </si>
+  <si>
+    <t>2026-07-04</t>
   </si>
 </sst>
 </file>
@@ -4016,4 +4344,1321 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I46"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E2" t="s">
+        <v>325</v>
+      </c>
+      <c r="F2" t="s">
+        <v>223</v>
+      </c>
+      <c r="G2">
+        <v>186</v>
+      </c>
+      <c r="H2">
+        <v>65000</v>
+      </c>
+      <c r="I2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>276</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" t="s">
+        <v>321</v>
+      </c>
+      <c r="E3" t="s">
+        <v>326</v>
+      </c>
+      <c r="F3" t="s">
+        <v>363</v>
+      </c>
+      <c r="G3">
+        <v>174</v>
+      </c>
+      <c r="H3">
+        <v>15000</v>
+      </c>
+      <c r="I3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D4" t="s">
+        <v>252</v>
+      </c>
+      <c r="E4" t="s">
+        <v>327</v>
+      </c>
+      <c r="F4" t="s">
+        <v>243</v>
+      </c>
+      <c r="G4">
+        <v>49</v>
+      </c>
+      <c r="H4">
+        <v>15000</v>
+      </c>
+      <c r="I4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>278</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D5" t="s">
+        <v>322</v>
+      </c>
+      <c r="E5" t="s">
+        <v>328</v>
+      </c>
+      <c r="F5" t="s">
+        <v>237</v>
+      </c>
+      <c r="G5">
+        <v>98</v>
+      </c>
+      <c r="H5">
+        <v>65000</v>
+      </c>
+      <c r="I5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>279</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>65</v>
+      </c>
+      <c r="D6" t="s">
+        <v>323</v>
+      </c>
+      <c r="E6" t="s">
+        <v>329</v>
+      </c>
+      <c r="F6" t="s">
+        <v>364</v>
+      </c>
+      <c r="G6">
+        <v>135</v>
+      </c>
+      <c r="H6">
+        <v>120000</v>
+      </c>
+      <c r="I6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>280</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>66</v>
+      </c>
+      <c r="E7" t="s">
+        <v>211</v>
+      </c>
+      <c r="F7" t="s">
+        <v>233</v>
+      </c>
+      <c r="G7">
+        <v>32</v>
+      </c>
+      <c r="H7">
+        <v>15000</v>
+      </c>
+      <c r="I7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>281</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" t="s">
+        <v>252</v>
+      </c>
+      <c r="E8" t="s">
+        <v>330</v>
+      </c>
+      <c r="F8" t="s">
+        <v>332</v>
+      </c>
+      <c r="G8">
+        <v>76</v>
+      </c>
+      <c r="H8">
+        <v>65000</v>
+      </c>
+      <c r="I8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>282</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" t="s">
+        <v>321</v>
+      </c>
+      <c r="E9" t="s">
+        <v>331</v>
+      </c>
+      <c r="F9" t="s">
+        <v>365</v>
+      </c>
+      <c r="G9">
+        <v>134</v>
+      </c>
+      <c r="H9">
+        <v>42000</v>
+      </c>
+      <c r="I9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>283</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" t="s">
+        <v>321</v>
+      </c>
+      <c r="E10" t="s">
+        <v>332</v>
+      </c>
+      <c r="F10" t="s">
+        <v>233</v>
+      </c>
+      <c r="G10">
+        <v>42</v>
+      </c>
+      <c r="H10">
+        <v>42000</v>
+      </c>
+      <c r="I10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>284</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" t="s">
+        <v>321</v>
+      </c>
+      <c r="E11" t="s">
+        <v>333</v>
+      </c>
+      <c r="H11">
+        <v>90000</v>
+      </c>
+      <c r="I11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>285</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" t="s">
+        <v>252</v>
+      </c>
+      <c r="E12" t="s">
+        <v>334</v>
+      </c>
+      <c r="F12" t="s">
+        <v>237</v>
+      </c>
+      <c r="G12">
+        <v>92</v>
+      </c>
+      <c r="H12">
+        <v>15000</v>
+      </c>
+      <c r="I12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>286</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D13" t="s">
+        <v>324</v>
+      </c>
+      <c r="E13" t="s">
+        <v>335</v>
+      </c>
+      <c r="F13" t="s">
+        <v>366</v>
+      </c>
+      <c r="G13">
+        <v>184</v>
+      </c>
+      <c r="H13">
+        <v>15000</v>
+      </c>
+      <c r="I13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>287</v>
+      </c>
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" t="s">
+        <v>61</v>
+      </c>
+      <c r="D14" t="s">
+        <v>323</v>
+      </c>
+      <c r="E14" t="s">
+        <v>336</v>
+      </c>
+      <c r="F14" t="s">
+        <v>367</v>
+      </c>
+      <c r="G14">
+        <v>140</v>
+      </c>
+      <c r="H14">
+        <v>65000</v>
+      </c>
+      <c r="I14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" t="s">
+        <v>288</v>
+      </c>
+      <c r="B15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" t="s">
+        <v>63</v>
+      </c>
+      <c r="D15" t="s">
+        <v>324</v>
+      </c>
+      <c r="E15" t="s">
+        <v>337</v>
+      </c>
+      <c r="F15" t="s">
+        <v>365</v>
+      </c>
+      <c r="G15">
+        <v>202</v>
+      </c>
+      <c r="H15">
+        <v>120000</v>
+      </c>
+      <c r="I15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" t="s">
+        <v>289</v>
+      </c>
+      <c r="B16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" t="s">
+        <v>324</v>
+      </c>
+      <c r="E16" t="s">
+        <v>337</v>
+      </c>
+      <c r="F16" t="s">
+        <v>327</v>
+      </c>
+      <c r="G16">
+        <v>202</v>
+      </c>
+      <c r="I16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" t="s">
+        <v>290</v>
+      </c>
+      <c r="B17" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" t="s">
+        <v>62</v>
+      </c>
+      <c r="D17" t="s">
+        <v>320</v>
+      </c>
+      <c r="E17" t="s">
+        <v>338</v>
+      </c>
+      <c r="F17" t="s">
+        <v>368</v>
+      </c>
+      <c r="G17">
+        <v>130</v>
+      </c>
+      <c r="H17">
+        <v>65000</v>
+      </c>
+      <c r="I17" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" t="s">
+        <v>291</v>
+      </c>
+      <c r="B18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" t="s">
+        <v>66</v>
+      </c>
+      <c r="D18" t="s">
+        <v>322</v>
+      </c>
+      <c r="E18" t="s">
+        <v>328</v>
+      </c>
+      <c r="F18" t="s">
+        <v>369</v>
+      </c>
+      <c r="G18">
+        <v>98</v>
+      </c>
+      <c r="H18">
+        <v>65000</v>
+      </c>
+      <c r="I18" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" t="s">
+        <v>292</v>
+      </c>
+      <c r="B19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19" t="s">
+        <v>339</v>
+      </c>
+      <c r="F19" t="s">
+        <v>370</v>
+      </c>
+      <c r="G19">
+        <v>167</v>
+      </c>
+      <c r="H19">
+        <v>90000</v>
+      </c>
+      <c r="I19" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" t="s">
+        <v>293</v>
+      </c>
+      <c r="B20" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" t="s">
+        <v>62</v>
+      </c>
+      <c r="D20" t="s">
+        <v>320</v>
+      </c>
+      <c r="E20" t="s">
+        <v>340</v>
+      </c>
+      <c r="F20" t="s">
+        <v>217</v>
+      </c>
+      <c r="G20">
+        <v>119</v>
+      </c>
+      <c r="H20">
+        <v>28000</v>
+      </c>
+      <c r="I20" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" t="s">
+        <v>294</v>
+      </c>
+      <c r="B21" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" t="s">
+        <v>68</v>
+      </c>
+      <c r="D21" t="s">
+        <v>324</v>
+      </c>
+      <c r="E21" t="s">
+        <v>203</v>
+      </c>
+      <c r="F21" t="s">
+        <v>204</v>
+      </c>
+      <c r="G21">
+        <v>19</v>
+      </c>
+      <c r="H21">
+        <v>28000</v>
+      </c>
+      <c r="I21" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" t="s">
+        <v>295</v>
+      </c>
+      <c r="B22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" t="s">
+        <v>252</v>
+      </c>
+      <c r="E22" t="s">
+        <v>341</v>
+      </c>
+      <c r="F22" t="s">
+        <v>217</v>
+      </c>
+      <c r="G22">
+        <v>109</v>
+      </c>
+      <c r="H22">
+        <v>90000</v>
+      </c>
+      <c r="I22" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" t="s">
+        <v>296</v>
+      </c>
+      <c r="B23" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" t="s">
+        <v>69</v>
+      </c>
+      <c r="D23" t="s">
+        <v>320</v>
+      </c>
+      <c r="E23" t="s">
+        <v>342</v>
+      </c>
+      <c r="F23" t="s">
+        <v>330</v>
+      </c>
+      <c r="G23">
+        <v>194</v>
+      </c>
+      <c r="H23">
+        <v>42000</v>
+      </c>
+      <c r="I23" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" t="s">
+        <v>297</v>
+      </c>
+      <c r="B24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" t="s">
+        <v>64</v>
+      </c>
+      <c r="D24" t="s">
+        <v>322</v>
+      </c>
+      <c r="E24" t="s">
+        <v>343</v>
+      </c>
+      <c r="H24">
+        <v>120000</v>
+      </c>
+      <c r="I24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" t="s">
+        <v>298</v>
+      </c>
+      <c r="B25" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" t="s">
+        <v>64</v>
+      </c>
+      <c r="D25" t="s">
+        <v>322</v>
+      </c>
+      <c r="E25" t="s">
+        <v>344</v>
+      </c>
+      <c r="F25" t="s">
+        <v>368</v>
+      </c>
+      <c r="G25">
+        <v>138</v>
+      </c>
+      <c r="H25">
+        <v>120000</v>
+      </c>
+      <c r="I25" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" t="s">
+        <v>299</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" t="s">
+        <v>62</v>
+      </c>
+      <c r="D26" t="s">
+        <v>323</v>
+      </c>
+      <c r="E26" t="s">
+        <v>345</v>
+      </c>
+      <c r="F26" t="s">
+        <v>229</v>
+      </c>
+      <c r="G26">
+        <v>90</v>
+      </c>
+      <c r="H26">
+        <v>42000</v>
+      </c>
+      <c r="I26" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" t="s">
+        <v>300</v>
+      </c>
+      <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" t="s">
+        <v>61</v>
+      </c>
+      <c r="D27" t="s">
+        <v>252</v>
+      </c>
+      <c r="E27" t="s">
+        <v>346</v>
+      </c>
+      <c r="F27" t="s">
+        <v>233</v>
+      </c>
+      <c r="G27">
+        <v>47</v>
+      </c>
+      <c r="H27">
+        <v>15000</v>
+      </c>
+      <c r="I27" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" t="s">
+        <v>301</v>
+      </c>
+      <c r="B28" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D28" t="s">
+        <v>252</v>
+      </c>
+      <c r="E28" t="s">
+        <v>347</v>
+      </c>
+      <c r="F28" t="s">
+        <v>371</v>
+      </c>
+      <c r="G28">
+        <v>207</v>
+      </c>
+      <c r="H28">
+        <v>15000</v>
+      </c>
+      <c r="I28" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" t="s">
+        <v>302</v>
+      </c>
+      <c r="B29" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29" t="s">
+        <v>68</v>
+      </c>
+      <c r="D29" t="s">
+        <v>324</v>
+      </c>
+      <c r="E29" t="s">
+        <v>348</v>
+      </c>
+      <c r="F29" t="s">
+        <v>372</v>
+      </c>
+      <c r="G29">
+        <v>102</v>
+      </c>
+      <c r="H29">
+        <v>15000</v>
+      </c>
+      <c r="I29" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" t="s">
+        <v>303</v>
+      </c>
+      <c r="B30" t="s">
+        <v>15</v>
+      </c>
+      <c r="C30" t="s">
+        <v>62</v>
+      </c>
+      <c r="D30" t="s">
+        <v>323</v>
+      </c>
+      <c r="E30" t="s">
+        <v>349</v>
+      </c>
+      <c r="F30" t="s">
+        <v>241</v>
+      </c>
+      <c r="G30">
+        <v>117</v>
+      </c>
+      <c r="H30">
+        <v>90000</v>
+      </c>
+      <c r="I30" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31" t="s">
+        <v>304</v>
+      </c>
+      <c r="B31" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31" t="s">
+        <v>63</v>
+      </c>
+      <c r="D31" t="s">
+        <v>322</v>
+      </c>
+      <c r="E31" t="s">
+        <v>350</v>
+      </c>
+      <c r="F31" t="s">
+        <v>371</v>
+      </c>
+      <c r="G31">
+        <v>159</v>
+      </c>
+      <c r="H31">
+        <v>15000</v>
+      </c>
+      <c r="I31" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" t="s">
+        <v>305</v>
+      </c>
+      <c r="B32" t="s">
+        <v>9</v>
+      </c>
+      <c r="C32" t="s">
+        <v>69</v>
+      </c>
+      <c r="E32" t="s">
+        <v>351</v>
+      </c>
+      <c r="F32" t="s">
+        <v>248</v>
+      </c>
+      <c r="G32">
+        <v>170</v>
+      </c>
+      <c r="H32">
+        <v>90000</v>
+      </c>
+      <c r="I32" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" t="s">
+        <v>306</v>
+      </c>
+      <c r="B33" t="s">
+        <v>14</v>
+      </c>
+      <c r="C33" t="s">
+        <v>68</v>
+      </c>
+      <c r="D33" t="s">
+        <v>321</v>
+      </c>
+      <c r="E33" t="s">
+        <v>352</v>
+      </c>
+      <c r="F33" t="s">
+        <v>227</v>
+      </c>
+      <c r="G33">
+        <v>91</v>
+      </c>
+      <c r="H33">
+        <v>42000</v>
+      </c>
+      <c r="I33" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" t="s">
+        <v>307</v>
+      </c>
+      <c r="B34" t="s">
+        <v>8</v>
+      </c>
+      <c r="C34" t="s">
+        <v>70</v>
+      </c>
+      <c r="D34" t="s">
+        <v>321</v>
+      </c>
+      <c r="E34" t="s">
+        <v>232</v>
+      </c>
+      <c r="F34" t="s">
+        <v>236</v>
+      </c>
+      <c r="G34">
+        <v>40</v>
+      </c>
+      <c r="H34">
+        <v>42000</v>
+      </c>
+      <c r="I34" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" t="s">
+        <v>308</v>
+      </c>
+      <c r="B35" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" t="s">
+        <v>63</v>
+      </c>
+      <c r="D35" t="s">
+        <v>320</v>
+      </c>
+      <c r="E35" t="s">
+        <v>353</v>
+      </c>
+      <c r="F35" t="s">
+        <v>329</v>
+      </c>
+      <c r="G35">
+        <v>156</v>
+      </c>
+      <c r="H35">
+        <v>28000</v>
+      </c>
+      <c r="I35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" t="s">
+        <v>309</v>
+      </c>
+      <c r="B36" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" t="s">
+        <v>68</v>
+      </c>
+      <c r="D36" t="s">
+        <v>252</v>
+      </c>
+      <c r="E36" t="s">
+        <v>329</v>
+      </c>
+      <c r="F36" t="s">
+        <v>373</v>
+      </c>
+      <c r="G36">
+        <v>135</v>
+      </c>
+      <c r="H36">
+        <v>15000</v>
+      </c>
+      <c r="I36" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" t="s">
+        <v>310</v>
+      </c>
+      <c r="B37" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" t="s">
+        <v>65</v>
+      </c>
+      <c r="D37" t="s">
+        <v>252</v>
+      </c>
+      <c r="E37" t="s">
+        <v>354</v>
+      </c>
+      <c r="F37" t="s">
+        <v>367</v>
+      </c>
+      <c r="G37">
+        <v>131</v>
+      </c>
+      <c r="H37">
+        <v>120000</v>
+      </c>
+      <c r="I37" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" t="s">
+        <v>311</v>
+      </c>
+      <c r="B38" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38" t="s">
+        <v>70</v>
+      </c>
+      <c r="D38" t="s">
+        <v>252</v>
+      </c>
+      <c r="E38" t="s">
+        <v>333</v>
+      </c>
+      <c r="F38" t="s">
+        <v>241</v>
+      </c>
+      <c r="G38">
+        <v>65</v>
+      </c>
+      <c r="H38">
+        <v>90000</v>
+      </c>
+      <c r="I38" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" t="s">
+        <v>312</v>
+      </c>
+      <c r="B39" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" t="s">
+        <v>65</v>
+      </c>
+      <c r="D39" t="s">
+        <v>323</v>
+      </c>
+      <c r="E39" t="s">
+        <v>355</v>
+      </c>
+      <c r="F39" t="s">
+        <v>248</v>
+      </c>
+      <c r="G39">
+        <v>33</v>
+      </c>
+      <c r="H39">
+        <v>28000</v>
+      </c>
+      <c r="I39" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" t="s">
+        <v>313</v>
+      </c>
+      <c r="B40" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" t="s">
+        <v>68</v>
+      </c>
+      <c r="D40" t="s">
+        <v>322</v>
+      </c>
+      <c r="E40" t="s">
+        <v>356</v>
+      </c>
+      <c r="F40" t="s">
+        <v>374</v>
+      </c>
+      <c r="G40">
+        <v>191</v>
+      </c>
+      <c r="I40" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" t="s">
+        <v>314</v>
+      </c>
+      <c r="B41" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" t="s">
+        <v>69</v>
+      </c>
+      <c r="D41" t="s">
+        <v>324</v>
+      </c>
+      <c r="E41" t="s">
+        <v>357</v>
+      </c>
+      <c r="F41" t="s">
+        <v>375</v>
+      </c>
+      <c r="G41">
+        <v>127</v>
+      </c>
+      <c r="H41">
+        <v>90000</v>
+      </c>
+      <c r="I41" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" t="s">
+        <v>315</v>
+      </c>
+      <c r="B42" t="s">
+        <v>14</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42" t="s">
+        <v>252</v>
+      </c>
+      <c r="E42" t="s">
+        <v>358</v>
+      </c>
+      <c r="F42" t="s">
+        <v>236</v>
+      </c>
+      <c r="G42">
+        <v>21</v>
+      </c>
+      <c r="H42">
+        <v>120000</v>
+      </c>
+      <c r="I42" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" t="s">
+        <v>316</v>
+      </c>
+      <c r="B43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C43" t="s">
+        <v>65</v>
+      </c>
+      <c r="D43" t="s">
+        <v>324</v>
+      </c>
+      <c r="E43" t="s">
+        <v>359</v>
+      </c>
+      <c r="F43" t="s">
+        <v>360</v>
+      </c>
+      <c r="G43">
+        <v>210</v>
+      </c>
+      <c r="H43">
+        <v>65000</v>
+      </c>
+      <c r="I43" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" t="s">
+        <v>317</v>
+      </c>
+      <c r="B44" t="s">
+        <v>15</v>
+      </c>
+      <c r="C44" t="s">
+        <v>65</v>
+      </c>
+      <c r="D44" t="s">
+        <v>322</v>
+      </c>
+      <c r="E44" t="s">
+        <v>360</v>
+      </c>
+      <c r="F44" t="s">
+        <v>376</v>
+      </c>
+      <c r="G44">
+        <v>164</v>
+      </c>
+      <c r="H44">
+        <v>120000</v>
+      </c>
+      <c r="I44" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" t="s">
+        <v>318</v>
+      </c>
+      <c r="B45" t="s">
+        <v>9</v>
+      </c>
+      <c r="C45" t="s">
+        <v>68</v>
+      </c>
+      <c r="D45" t="s">
+        <v>320</v>
+      </c>
+      <c r="E45" t="s">
+        <v>361</v>
+      </c>
+      <c r="F45" t="s">
+        <v>248</v>
+      </c>
+      <c r="G45">
+        <v>100</v>
+      </c>
+      <c r="H45">
+        <v>120000</v>
+      </c>
+      <c r="I45" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" t="s">
+        <v>319</v>
+      </c>
+      <c r="B46" t="s">
+        <v>10</v>
+      </c>
+      <c r="C46" t="s">
+        <v>66</v>
+      </c>
+      <c r="D46" t="s">
+        <v>320</v>
+      </c>
+      <c r="E46" t="s">
+        <v>362</v>
+      </c>
+      <c r="F46" t="s">
+        <v>368</v>
+      </c>
+      <c r="G46">
+        <v>141</v>
+      </c>
+      <c r="H46">
+        <v>120000</v>
+      </c>
+      <c r="I46" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>